<commit_message>
more toasts for send to qc
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/dist/release/Full-LC-AUTO/successful-run-record.xlsx
+++ b/Full-LC-AUTO/dist/release/Full-LC-AUTO/successful-run-record.xlsx
@@ -395,7 +395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,6 +459,16 @@
           <t>2026-07-08</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
@@ -513,6 +523,16 @@
           <t>Seema</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Prabhu</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Seema</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -540,6 +560,11 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>2-FADE 5-IND</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>1-STAR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added queuing in full lc auto
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/dist/release/Full-LC-AUTO/successful-run-record.xlsx
+++ b/Full-LC-AUTO/dist/release/Full-LC-AUTO/successful-run-record.xlsx
@@ -395,7 +395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,16 @@
           <t>2026-07-09</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
@@ -533,6 +543,16 @@
           <t>Seema</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Prabhu</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Seema</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -737,6 +757,23 @@
       <c r="K15" t="inlineStr">
         <is>
           <t>1-GENZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Track Pant</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>flipkart</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>1-STAR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NEW PRINTER MIDDLEWARE FOR ORDER SORTING
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/dist/release/Full-LC-AUTO/successful-run-record.xlsx
+++ b/Full-LC-AUTO/dist/release/Full-LC-AUTO/successful-run-record.xlsx
@@ -395,7 +395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:R17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,6 +479,16 @@
           <t>2026-07-18</t>
         </is>
       </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
@@ -553,6 +563,16 @@
           <t>Seema</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Prabhu</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Seema</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -774,6 +794,23 @@
       <c r="O16" t="inlineStr">
         <is>
           <t>2-STAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>White-Baggy</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>flipkart</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1-STAR</t>
         </is>
       </c>
     </row>

</xml_diff>